<commit_message>
Park hours: Otter Creek fee + hours from KDFWR's brochure (Brandon caught the miss)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015sd9rGiF55g53SvUATRP26
</commit_message>
<xml_diff>
--- a/.claude/build/research/KPC_Park_Hours_done.xlsx
+++ b/.claude/build/research/KPC_Park_Hours_done.xlsx
@@ -7793,7 +7793,7 @@
       </c>
       <c r="E179" s="8" t="inlineStr">
         <is>
-          <t>Open year-round from dawn to dusk.</t>
+          <t>Wednesday-Sunday, daylight to dark; closed Monday and Tuesday</t>
         </is>
       </c>
       <c r="F179" s="8" t="inlineStr">
@@ -7801,15 +7801,19 @@
           <t>General area closes at dusk; campground is operated separately by Meade County Fiscal Court. Overnight rules for campground are managed by the county.</t>
         </is>
       </c>
-      <c r="G179" s="8" t="n"/>
+      <c r="G179" s="8" t="inlineStr">
+        <is>
+          <t>$3.00 per person per day ($30.00 a year); under 12 free; trails/shooting range +$7.00 a day ($70.00 a year)</t>
+        </is>
+      </c>
       <c r="H179" s="8" t="inlineStr">
         <is>
-          <t>https://fw.ky.gov/Pages/Otter-Creek-Outdoor-Recreation-Area.aspx</t>
+          <t>https://fw.ky.gov/Documents/ottercreekbrochure.pdf</t>
         </is>
       </c>
       <c r="I179" s="8" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>DONE (fixed by HQ Oct 25 from KDFWR brochure; entry permit required by 301 KAR 3:012)</t>
         </is>
       </c>
     </row>

</xml_diff>